<commit_message>
Commiting the changes for testplans execution
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated_TC6.xlsx
+++ b/uploads/Bid_file_success_error_newly_updated_TC6.xlsx
@@ -542,7 +542,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TestSigma_03-04-2026_SC1_u1_393</v>
+        <v>TestSigma_04-05-2026_SC1_8h_695</v>
       </c>
       <c r="B2">
         <v>2001</v>
@@ -656,7 +656,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TestSigma_03-04-2026_SC1_7g_734</v>
+        <v>TestSigma_04-05-2026_SC1_vv_514</v>
       </c>
       <c r="B3">
         <v>2001</v>
@@ -770,7 +770,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>TestSigma_03-04-2026_SC1_ap_289</v>
+        <v>TestSigma_04-05-2026_SC1_pg_182</v>
       </c>
       <c r="B4">
         <v>2001</v>
@@ -883,7 +883,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>TestSigma_03-04-2026_SC1_sd_242</v>
+        <v>TestSigma_04-05-2026_SC1_4o_442</v>
       </c>
       <c r="B5">
         <v>2001</v>
@@ -996,7 +996,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>TestSigma_03-04-2026_SC1_lu_923</v>
+        <v>TestSigma_04-05-2026_SC1_zq_557</v>
       </c>
       <c r="B6">
         <v>2001</v>
@@ -1109,7 +1109,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>TestSigma_03-04-2026_SC1_b3_772</v>
+        <v>TestSigma_04-05-2026_SC1_q5_105</v>
       </c>
       <c r="B7">
         <v>2001</v>

</xml_diff>